<commit_message>
Sprint 67 (M6): candidate parity on the phone (ADR-078, BL-15.9 to BL-15.11)
The phone gains what the website's candidate already had: the six profile
history sections through one table-driven editor (limits compared with the
server's schema by tests/test_mobile_section_limits.py), "why not me" on a
rejected application, career paths, a device-held course budget forgotten at
sign-out, and salary/notice/work-type/relocation/alert preferences. Date of
birth and gender stay web-only. No migration, no new endpoint: five existing
operations join the released surface (46 to 51, additive).

Housekeeping: ADR-019/032/033/037 headers say what superseded them,
scripts/build_adr_register.py rebuilds the ADR register (tests fail when it is
stale), backlog v1.28.

Browser-run in both languages; not run on a device.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/adr/IISM-ADR-Register.xlsx
+++ b/docs/adr/IISM-ADR-Register.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 63 of 77 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file was kept up to date through ADR-077 (this sprint).</t>
+          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 64 of 78 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-078.</t>
         </is>
       </c>
     </row>
@@ -165,7 +165,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No. 7 ADRs are formally superseded (whole or in part), 3 are only partly built, 2 are not built, 2 are deferred by the owner. Four headers (ADR-019, 032, 033, 037) still read plain 'Accepted' although a later ADR or event changed their meaning (see 'Stale headers').</t>
+          <t xml:space="preserve">No. 7 ADRs are formally superseded (whole or in part), 3 are only partly built, 2 are not built, 2 are deferred by the owner. Four headers (ADR-019, 032, 033, 037) that once read plain 'Accepted' although a later ADR or event had changed their meaning now say so (Sprint 67); 'Stale headers' lists the decisions whose header says nothing of how far they are built.</t>
         </is>
       </c>
     </row>
@@ -177,7 +177,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No. A rewrite would lose the reasoning and the trade-offs, which are the point of an ADR. Recommended: a one-line status edit on four headers, and keep this register as the shareable index.</t>
+          <t xml:space="preserve">No. A rewrite would lose the reasoning and the trade-offs, which are the point of an ADR. Keep this register as the shareable index, and regenerate it with scripts/build_adr_register.py when an ADR is added.</t>
         </is>
       </c>
     </row>
@@ -225,7 +225,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">From docs/adr/architecture-decisions.md at the Sprint 66 commit (c7c7d7c).</t>
+          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit f4e0313 by scripts/build_adr_register.py.</t>
         </is>
       </c>
     </row>
@@ -261,7 +261,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">63</t>
+          <t xml:space="preserve">64</t>
         </is>
       </c>
     </row>
@@ -1767,12 +1767,12 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted</t>
+          <t xml:space="preserve">Accepted. Superseded in part by ADR-040 (the tooling: structured JSON logs to stdout). OpenTelemetry, Prometheus and Grafana remain the destination and are deferred, not built.</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ADR-040</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -2703,12 +2703,12 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted (September 2026)</t>
+          <t xml:space="preserve">Accepted (September 2026). Superseded in part by ADR-038 (the organisation half: email one-time code, no password). The rule that a candidate signs up by phone still governs.</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ADR-038</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
@@ -2775,12 +2775,12 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted (September 2026)</t>
+          <t xml:space="preserve">Accepted (September 2026). Superseded in part by ADR-041 (the two-language assumption: a language is a messages file and rows). Hindi and English remain the launch pair.</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ADR-041</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
@@ -3063,12 +3063,12 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted (September 2026)</t>
+          <t xml:space="preserve">Accepted (September 2026). Superseded in part by ADR-038 (the authenticated employer console ships to production, behind a sign-in). The rule that no employer-facing payload identifies a candidate stands and is tested; only the unauthenticated demonstration console is local-only.</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ADR-038</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -5967,8 +5967,80 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-078</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Phone Holds No Data the Website Does Not, Edits a History Section Through One Table Checked Against the Schema, and Keeps a Course Budget Only on the Device and Only Until Sign-Out</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">October 2026</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">67</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Active – extends earlier ADR</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Built</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- A phone adds no data type the website does not hold. The Data Safety and App Privacy answers (docs/release/privacy-and-data-safety.md) are unchanged. Date of birth and gender stay web-only: they are optional and sensitive, nothing on the phone needs them, and a phone is the device most likely to be shared. A person's salary range, notice period, work type, willingness to move and alert opt-out are the same…</t>
+        </is>
+      </c>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted (October 2026). Sprint 67 (BL-15.9 to BL-15.11, M6 of the mobile programme). Extends ADR-048, ADR-049, ADR-068, ADR-072 and ADR-074. No migration, no new endpoint: five operations that the website already calls join the released surface (46 to 51, additive only).</t>
+        </is>
+      </c>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-048, ADR-049, ADR-068, ADR-072, ADR-074</t>
+        </is>
+      </c>
+      <c r="L79" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint 67 (M6). Candidate parity on the phone: history sections, why-not-me, careers, budget. Tested and browser-run; not run on a device.</t>
+        </is>
+      </c>
+      <c r="N79" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR header and sprint record in CLAUDE.md / projectContextForMe.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N78"/>
+  <autoFilter ref="A1:N79"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
@@ -6015,7 +6087,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADR-019 Observability Strategy</t>
+          <t xml:space="preserve">ADR-005 AI Strategy</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -6025,105 +6097,105 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tooling half replaced by ADR-040 (structured JSON logs to stdout). The destination (OpenTelemetry, Prometheus, Grafana) remains deferred and unbuilt.</t>
+          <t xml:space="preserve">No LLM call exists anywhere; the intelligence/ module has an ADR and no code. The direction stands: ADR-036 keeps every decision deterministic and lets a model only explain.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Header silent about a later ADR or event</t>
+          <t xml:space="preserve">Decision stands; header says nothing of implementation lag</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Superseded in part by ADR-040 (tooling); destination deferred.</t>
+          <t xml:space="preserve">Accepted; not built.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADR-032 Primary Credential by Actor Type</t>
+          <t xml:space="preserve">ADR-011 Identity Model</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted (September 2026)</t>
+          <t xml:space="preserve">Accepted</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The organisation half (email OTP, password-free) is replaced by ADR-038; the credential-follows-actor rule still governs sign-up.</t>
+          <t xml:space="preserve">UUID primary key built. Optional Aadhaar verification is not built and nothing collects Aadhaar data.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Header silent about a later ADR or event</t>
+          <t xml:space="preserve">Decision stands; header says nothing of implementation lag</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Superseded in part by ADR-038 (organisation half).</t>
+          <t xml:space="preserve">Accepted; Aadhaar verification not built.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADR-033 Language Scope at Launch</t>
+          <t xml:space="preserve">ADR-013 Embedding Strategy</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted (September 2026)</t>
+          <t xml:space="preserve">Accepted</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The two-language assumption is replaced by ADR-041 (a language is a messages file and rows). Hindi and English remain the launch pair; Malay is hidden from the switcher, not removed.</t>
+          <t xml:space="preserve">pgvector storage and a 384-dimension port are built (ADR-031). The mandated sentence-transformers model is not switched on: HashingEmbeddingProvider is an honest placeholder and BL-5.3 is not started.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Header silent about a later ADR or event</t>
+          <t xml:space="preserve">Decision stands; header says nothing of implementation lag</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Superseded in part by ADR-041 (two-language assumption).</t>
+          <t xml:space="preserve">Accepted; placeholder embedder in use (BL-5.3).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADR-037 The Employer Console as a Labelled Demonstration</t>
+          <t xml:space="preserve">ADR-018 AI Model Strategy</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted (September 2026)</t>
+          <t xml:space="preserve">Accepted</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The rule that no employer-facing payload identifies a candidate stands and is tested. The 'unauthenticated demonstration' framing no longer describes the product: the authenticated employer console shipped to production in Sprint 12 (ADR-038); only the unauthenticated demo console is local-only.</t>
+          <t xml:space="preserve">No external LLM is integrated. The adapter pattern it depends on exists (ADR-017, ADR-031).</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Header silent about a later ADR or event</t>
+          <t xml:space="preserve">Decision stands; header says nothing of implementation lag</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Superseded in part: console is authenticated and ships to production (ADR-038); de-identification rule stands.</t>
+          <t xml:space="preserve">Accepted; not built.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADR-005 AI Strategy</t>
+          <t xml:space="preserve">ADR-023 Data Privacy &amp; Compliance</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -6133,7 +6205,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No LLM call exists anywhere; the intelligence/ module has an ADR and no code. The direction stands: ADR-036 keeps every decision deterministic and lets a model only explain.</t>
+          <t xml:space="preserve">Consent record, DPDP export, erasure, the redaction filter and retention are built. The encryption path for Aadhaar, resumes and assessment results is not, so that data is deliberately not collected.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -6143,24 +6215,24 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted; not built.</t>
+          <t xml:space="preserve">Accepted; encryption path unbuilt.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADR-011 Identity Model</t>
+          <t xml:space="preserve">ADR-025 Monetization Model</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted</t>
+          <t xml:space="preserve">Accepted (September 2026)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">UUID primary key built. Optional Aadhaar verification is not built and nothing collects Aadhaar data.</t>
+          <t xml:space="preserve">Monetisation (BL-1.3) is a standing not-started: the owner chose to wait for real traffic. ADR-043 and ADR-047 carry the deferral.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -6170,24 +6242,24 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted; Aadhaar verification not built.</t>
+          <t xml:space="preserve">Accepted; deferred by owner.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADR-013 Embedding Strategy</t>
+          <t xml:space="preserve">ADR-028 Cloud Platform and Deployment Topology</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted</t>
+          <t xml:space="preserve">Accepted (September 2026)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">pgvector storage and a 384-dimension port are built (ADR-031). The mandated sentence-transformers model is not switched on: HashingEmbeddingProvider is an honest placeholder and BL-5.3 is not started.</t>
+          <t xml:space="preserve">Nothing is deployed anywhere; deployment is deferred by the owner and is now on the mobile launch's critical path. Still the intended topology.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -6197,120 +6269,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted; placeholder embedder in use (BL-5.3).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ADR-018 AI Model Strategy</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Accepted</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No external LLM is integrated. The adapter pattern it depends on exists (ADR-017, ADR-031).</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Decision stands; header says nothing of implementation lag</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Accepted; not built.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ADR-023 Data Privacy &amp; Compliance</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Accepted</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Consent record, DPDP export, erasure, the redaction filter and retention are built. The encryption path for Aadhaar, resumes and assessment results is not, so that data is deliberately not collected.</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Decision stands; header says nothing of implementation lag</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Accepted; encryption path unbuilt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ADR-025 Monetization Model</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Accepted (September 2026)</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Monetisation (BL-1.3) is a standing not-started: the owner chose to wait for real traffic. ADR-043 and ADR-047 carry the deferral.</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Decision stands; header says nothing of implementation lag</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Accepted; deferred by owner.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ADR-028 Cloud Platform and Deployment Topology</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Accepted (September 2026)</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nothing is deployed anywhere; deployment is deferred by the owner and is now on the mobile launch's critical path. Still the intended topology.</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Decision stands; header says nothing of implementation lag</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
           <t xml:space="preserve">Accepted; deferred by owner, nothing deployed.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E12"/>
+  <autoFilter ref="A1:E8"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
@@ -6810,8 +6774,30 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint 67</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-078</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Phone Holds No Data the Website Does Not, Edits a History Section Through One Table Checked Against the Schema, and Keeps a Course Budget Only on the Device and Only Until Sign-Out</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D22"/>
+  <autoFilter ref="A1:D23"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Sprint 69: scannable jobs (BL-16.1, ADR-079)
Cards say what, who, where, pay a month and when it closes (a verified mark,
never "not verified" on a card; no NSQF badge or generated sentence). Pay is
monthly via a rule shared by web and phone and tested against one fixture file.
/jobs and /courses page 24 at a time with the server's total; new
GET /jobs/states is the state filter. Apply bar follows the thumb (web and
phone), standards are deduplicated and sentence-cased, a trust strip is added,
nothing is under 12 px, header/footer/buttons are 44 px (asserted in the browser
sweep), and both operator queues return {items, total}.

Measured with the review's script: /jobs 42.3 -> 7.5 screens, text under 12 px
296 -> 0. 1,835 backend / 615 web / 649 mobile / 130 browser tests; 37 mutants.
No migration. Not user research, not run on a device.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/adr/IISM-ADR-Register.xlsx
+++ b/docs/adr/IISM-ADR-Register.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 64 of 78 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-078.</t>
+          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 65 of 79 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-079.</t>
         </is>
       </c>
     </row>
@@ -225,7 +225,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit 4477bef by scripts/build_adr_register.py.</t>
+          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit 6411ef6 by scripts/build_adr_register.py.</t>
         </is>
       </c>
     </row>
@@ -261,7 +261,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">64</t>
+          <t xml:space="preserve">65</t>
         </is>
       </c>
     </row>
@@ -6039,8 +6039,80 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-079</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A Listing Says What Decides Whether to Open It in the Units People Use, a Rule Both Clients Share Is Tested Against One File, a Count Comes From the Server, and Touch and Type Have Floors a Browser Test Holds</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">October 2026</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">69</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Active – extends earlier ADR</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Built</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- A card carries what decides whether to open it, in the order people ask: what, who, where, how much, by when. The employer carries a verified mark when it has earned one; a card never says "not verified", because in a list the absence of a mark would read as an accusation of every employer without one, and the vacancy's own page is where "not yet verified" and "never pay to apply" are stated. The NSQF level and…</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted (October 2026). Sprint 69 (BL-16.1, from the UI review of Sprint 68). Extends ADR-037, ADR-065, ADR-068, ADR-072 and ADR-074. No migration. One endpoint is new (GET /jobs/states, public, additive) and the two operator queues change shape (/ops/organisations and /ops/candidates/certifications return {items, total, limit, offset}); neither is in the released mobile surface, which stays at 51.</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-037, ADR-065, ADR-068, ADR-072, ADR-074</t>
+        </is>
+      </c>
+      <c r="L80" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint 69 (BL-16.1). Scannable listings: monthly pay, card v2, server totals, a shared fixture for rules both clients need, 12 px and 44 px floors held by tests.</t>
+        </is>
+      </c>
+      <c r="N80" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR header and sprint record in CLAUDE.md / projectContextForMe.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N79"/>
+  <autoFilter ref="A1:N80"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
@@ -6796,8 +6868,30 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint 69</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-079</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A Listing Says What Decides Whether to Open It in the Units People Use, a Rule Both Clients Share Is Tested Against One File, a Count Comes From the Server, and Touch and Type Have Floors a Browser Test Holds</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D23"/>
+  <autoFilter ref="A1:D24"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Sprint 71: role search you can trust (BL-12.12, ADR-081)
Role-alias coverage goes from 114 forms onto 41 roles to 307 onto 88
(English, romanised Hindi, Devanagari), every target a general pack and
checked against the real corpus. Measured for the first time by
`make evaluate-roles` over 146 titles written before any alias, a third
held out: tuning top-1 76.5% -> 99.0%, all 65.5% -> 81.7%, hold-out
unchanged at 37.5% (aliases cover only the words they name).

- scripts/evaluate_role_search.py, tests/fixtures/role_titles.json and a
  static guard (tests/test_role_titles.py) for CI
- docs/IISM-Role-Aliases-for-Review.xlsx built from the dict, with a
  staleness test; the batch is an unreviewed engineering draft
- no ranking change, no migration, no new operation
- role_aliases.py docstring corrected (waiter and mason do have packs)
- ADR-081, register, backlog v1.32, CLAUDE.md, projectContextForMe.md

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/adr/IISM-ADR-Register.xlsx
+++ b/docs/adr/IISM-ADR-Register.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 66 of 80 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-080.</t>
+          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 67 of 81 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-081.</t>
         </is>
       </c>
     </row>
@@ -225,7 +225,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit 021c147 by scripts/build_adr_register.py.</t>
+          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit c373a5d by scripts/build_adr_register.py.</t>
         </is>
       </c>
     </row>
@@ -261,7 +261,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">66</t>
+          <t xml:space="preserve">67</t>
         </is>
       </c>
     </row>
@@ -6183,8 +6183,80 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-081</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Role-Search Vocabulary Is Measured Against Titles Written Before It, a Hold-Out Is Reported Separately, and an Unreviewed Draft Says So Where a Reviewer Will Find It</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">October 2026</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">71</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Active – extends earlier ADR</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Built</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- Titles are written before the aliases and not from what search answers. tests/fixtures/role_titles.json holds 146 titles people say (118 English, 12 romanised Hindi, 16 Devanagari) across the sectors. Each carries the corpus roles that honestly fit, chosen by meaning from a listing of the corpus (an exact name, or a case-insensitive pattern over role names), or none_ok for a job the corpus has no role for, with…</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted (October 2026). Sprint 71 (BL-12.12). Extends ADR-050 and ADR-054. No migration, no new operation (the released surface stays at 51), and no ranking change.</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-050, ADR-054</t>
+        </is>
+      </c>
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint 71 (BL-12.12). Role-alias coverage 41 to 88 roles, measured against titles written first; the hold-out did not move (37.5%) and is reported. Unreviewed draft, flagged.</t>
+        </is>
+      </c>
+      <c r="N82" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR header and sprint record in CLAUDE.md / projectContextForMe.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N81"/>
+  <autoFilter ref="A1:N82"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
@@ -6984,8 +7056,30 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint 71</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-081</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Role-Search Vocabulary Is Measured Against Titles Written Before It, a Hold-Out Is Reported Separately, and an Unreviewed Draft Says So Where a Reviewer Will Find It</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D25"/>
+  <autoFilter ref="A1:D26"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Sprint 77: Epic B19 foundations - colour ramps, type scale, shape tokens (ADR-086)
BL-19.4, BL-19.5, BL-19.6. Brand and tinted neutral ramps as variables with
semantic tokens re-pointed (grey page, white cards); a six-step named type
scale (secondary text 15 px, 12 px floor) mapped onto Tailwind's text names
with taller Devanagari line heights; radii 6/10/16, card shadow, motion and a
reduced-motion rule. The mobile token sync now emits radius and type without
treating them as colours. 93 new token tests (contrast of every pairing in
both themes) and a guard that forbids translucent text, which the browser run
found failing contrast in dark (CTA band, footer). Frontend only: no
migration, no API or contract change.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/adr/IISM-ADR-Register.xlsx
+++ b/docs/adr/IISM-ADR-Register.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 71 of 85 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-085.</t>
+          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 72 of 86 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-086.</t>
         </is>
       </c>
     </row>
@@ -225,7 +225,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit b7d69ab by scripts/build_adr_register.py.</t>
+          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit 3b57ff6 by scripts/build_adr_register.py.</t>
         </is>
       </c>
     </row>
@@ -261,7 +261,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">71</t>
+          <t xml:space="preserve">72</t>
         </is>
       </c>
     </row>
@@ -6543,8 +6543,80 @@
         </is>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-086</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Look Is Chosen in One Place: Colour Ramps, a Named Type Scale and Shape Tokens in `globals.css`, Generated Into the Phone; a Ramp Step Is Never a Class, and Text Is Never Translucent</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">October 2026</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">77</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Active – extends earlier ADR</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Built</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- Two ramps, defined once. --brand-50 to --brand-900 (700 is today's #1f4e79; the dark theme's primary is 400) and --neutral-50 to --neutral-950 (tinted to the brand hue), as variables in globals.css. The semantic tokens (background, surface, border, control edge, muted text, brand, the four tones) are re-pointed at steps in both themes. The page is neutral-50 and a card is white, so a card is a surface instead…</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted (October 2026). Sprint 77 (Epic B19, BL-19.4, BL-19.5, BL-19.6). Extends ADR-065 (a page must not jump while it loads; the Hindi fold is a budget), ADR-077 (accessibility is held by the props that produce it) and ADR-079 (floors are asserted where they hold for every page); implements the direction the Product Owner signed off in docs/design/design-brief.md (Sprint 76). Frontend only: no migration, no API or contract change, the released surface stays at 54 operations.</t>
+        </is>
+      </c>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-065, ADR-077, ADR-079</t>
+        </is>
+      </c>
+      <c r="L87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR header and sprint record in CLAUDE.md / projectContextForMe.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N86"/>
+  <autoFilter ref="A1:N87"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
@@ -7454,8 +7526,30 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint 77</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-086</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Look Is Chosen in One Place: Colour Ramps, a Named Type Scale and Shape Tokens in `globals.css`, Generated Into the Phone; a Ramp Step Is Never a Class, and Text Is Never Translucent</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D30"/>
+  <autoFilter ref="A1:D31"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Sprint 78: Epic B19 foundations complete - icons, guards, theme control (ADR-087)
BL-19.7, BL-19.9, BL-19.8. 34 icons drawn once on the web, imported one at a
time (the header graph imports none: it cost /profile 863 B), the phone's
shapes generated from them. Ratchets that only go down: a recorded count of
controls under 44 px per sweep page, token adoption for migrated families,
and layout-shift scoring in the phone's browser run (which found the
signed-in home jumping, recorded as a known ceiling for BL-19.22). Light,
dark or the device on the web (head script before first paint, closed footer
disclosure loaded on first open: /profile +410 B) and the phone (chips on Me,
forgotten at sign-out). Frontend only: no migration, no API or contract change.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/adr/IISM-ADR-Register.xlsx
+++ b/docs/adr/IISM-ADR-Register.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 72 of 86 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-086.</t>
+          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 73 of 87 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-087.</t>
         </is>
       </c>
     </row>
@@ -225,7 +225,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit 3b57ff6 by scripts/build_adr_register.py.</t>
+          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit 1fabbae by scripts/build_adr_register.py.</t>
         </is>
       </c>
     </row>
@@ -261,7 +261,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">72</t>
+          <t xml:space="preserve">73</t>
         </is>
       </c>
     </row>
@@ -6615,8 +6615,80 @@
         </is>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-087</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Icons Are Drawn Once and Imported One at a Time, the Revamp Is Held by Ratchets That Only Go Down, and a Person May Choose Light or Dark Without the First Load Paying for It</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">October 2026</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">78</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Active – extends earlier ADR</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Built</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- Thirty-four icons, drawn once, imported one at a time. web/src/components/ui/icons.tsx holds makeIcon("Name", [paths]) calls, each marked /#__PURE__/, on a 24 grid with a 2 px round stroke in currentColor: no package, no image request, no download. Each icon is its own export so a route pays only for the icons it imports; a table looked up by name would put every shape on every route. An icon beside its word is…</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted (October 2026). Sprint 78 (Epic B19, BL-19.7 icon set, BL-19.9 guards for the revamp, BL-19.8 theme control). Extends ADR-086 (tokens), ADR-065 (a page must not jump while it loads), ADR-077 (accessibility is held by the props that produce it) and ADR-079 (floors are asserted where they hold for every page). Frontend only: no migration, no API or contract change, the released surface stays at 54 operations.</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-065, ADR-077, ADR-079, ADR-086</t>
+        </is>
+      </c>
+      <c r="L88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR header and sprint record in CLAUDE.md / projectContextForMe.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N87"/>
+  <autoFilter ref="A1:N88"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
@@ -7548,8 +7620,30 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint 78</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-087</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Icons Are Drawn Once and Imported One at a Time, the Revamp Is Held by Ratchets That Only Go Down, and a Person May Choose Light or Dark Without the First Load Paying for It</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D31"/>
+  <autoFilter ref="A1:D32"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Sprint 79: form controls with inline validation (ADR-088)
BL-19.10. One field library (label tied by htmlFor, hint, problem slot,
aria-describedby and aria-invalid by context, 44 px) re-exported under the
old profile helper names, so 25 forms keep their markup and literal limits.
A problem shows beside its field when the person leaves it, in the page's
words; where the server refused, its own words land beside the field it
named (ApiError.fields; all 64 hand-built ApiErrors now go through
apiErrorFrom). The checks and the profile sections' fields load on first
use: /profile is 2,617 B under where the sprint began (headroom 5,444).
Frontend only: no migration, no API or contract change.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/adr/IISM-ADR-Register.xlsx
+++ b/docs/adr/IISM-ADR-Register.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 73 of 87 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-087.</t>
+          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 74 of 88 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-088.</t>
         </is>
       </c>
     </row>
@@ -225,7 +225,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit 1fabbae by scripts/build_adr_register.py.</t>
+          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit f32ae25 by scripts/build_adr_register.py.</t>
         </is>
       </c>
     </row>
@@ -261,7 +261,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">73</t>
+          <t xml:space="preserve">74</t>
         </is>
       </c>
     </row>
@@ -6687,8 +6687,80 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-088</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A Form Field Says What Is Wrong Next to Itself, in the Page's Words or the Server's; the Library's Controls Are the Old Helpers Under the Same Names, and What a Form Does Not Need at First Paint Is Fetched When It Is Opened</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">October 2026</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">79</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Active – extends earlier ADR</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Built</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- One library, components/ui/field.tsx, and the old names stay. Field (label, hint, problem), Input, Textarea, Select and Checkbox; components/profile/fields.tsx re-exports them as Field, Text, Area, Select, Check, so the 25 forms that use them changed none of their markup and the limits (minLength={3}) stay literal at each control where constraints.test.ts reads them. Field provides a context; the control reads…</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted (October 2026). Sprint 79 (Epic B19, BL-19.10, first half: the library, the validation and the four forms that matter most; the other raw controls move in the page-family stories). Extends ADR-086 (tokens), ADR-087 (ratchets, the header graph and the first-load budget) and the Sprint 29 and 30 conventions that a form mirrors the server's limits and never throws away what the server said. Frontend only: no migration, no API or contract change (54 operations).</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-086, ADR-087</t>
+        </is>
+      </c>
+      <c r="L89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR header and sprint record in CLAUDE.md / projectContextForMe.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N88"/>
+  <autoFilter ref="A1:N89"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
@@ -7642,8 +7714,30 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint 79</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-088</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A Form Field Says What Is Wrong Next to Itself, in the Page's Words or the Server's; the Library's Controls Are the Old Helpers Under the Same Names, and What a Form Does Not Need at First Paint Is Fetched When It Is Opened</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D32"/>
+  <autoFilter ref="A1:D33"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Sprint 80: surfaces, actions and empty/status states (ADR-089)
BL-19.11, BL-19.12. Card levels (default, raised, inset for a box in a card,
interactive), badge sizes and an info tone, button soft/pressed/loading
variants, and alerts that draw a shape per tone (written inline, held equal
to the icon set by a test). One EmptyState (icon, sentence, action, slot for
art) in ten empty lists, a Spinner, and no toast. A dev-only /gallery,
present only in the browser-test build, is swept in en, hi and on a phone
with contrast checked in light and dark. Barrel exports of EmptyState and
Spinner cost /profile 4,124 B and were removed (tested); /profile ends 1,659 B
above where the sprint began (headroom 3,785). Frontend only: no migration,
no API or contract change.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/adr/IISM-ADR-Register.xlsx
+++ b/docs/adr/IISM-ADR-Register.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 74 of 88 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-088.</t>
+          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 75 of 89 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-089.</t>
         </is>
       </c>
     </row>
@@ -225,7 +225,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit f32ae25 by scripts/build_adr_register.py.</t>
+          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit b83d88e by scripts/build_adr_register.py.</t>
         </is>
       </c>
     </row>
@@ -261,7 +261,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">74</t>
+          <t xml:space="preserve">75</t>
         </is>
       </c>
     </row>
@@ -6759,8 +6759,80 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-089</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A Card Has a Level, a Status Has a Shape, an Empty List Has an Icon and a Slot for Art, and a Gallery Shows Them All in a Build That Is Never Shipped</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">October 2026</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">80</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Active – extends earlier ADR</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Built</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- A card has a level. Card level="default | raised | inset | interactive": the default is what it always was plus the soft shadow (the page is grey and a card is white, ADR-086), raised is the floating surface (a menu, a dialog's panel), inset is a box inside a card (the muted surface, no shadow: a bordered, shadowed card in a card was how a form held a sub-panel), and interactive lifts on hover and takes the…</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted (October 2026). Sprint 80 (Epic B19, BL-19.11 surfaces and actions, BL-19.12 empty, loading and status states). Extends ADR-086 (tokens), ADR-087 (the icon set, the header graph and the first-load budget) and ADR-088 (the form library). Frontend only: no migration, no API or contract change (54 operations).</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-086, ADR-087, ADR-088</t>
+        </is>
+      </c>
+      <c r="L90" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N90" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR header and sprint record in CLAUDE.md / projectContextForMe.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N89"/>
+  <autoFilter ref="A1:N90"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
@@ -7736,8 +7808,30 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint 80</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-089</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A Card Has a Level, a Status Has a Shape, an Empty List Has an Icon and a Slot for Art, and a Gallery Shows Them All in a Build That Is Never Shipped</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D33"/>
+  <autoFilter ref="A1:D34"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Sprint 81: header, footer and navigation (ADR-090)
BL-19.13. The current page is marked in the header (longest matching link,
aria-current); sign-in and sign-up get a reduced header; the mobile menu
closes on Escape or a tap outside and scrolls inside the screen. A job
seeker's own pages (matches, applications, saved jobs, updates, profile,
courses asked about, career paths, account) are a row at the top of each of
them. On a phone's browser a signed-in seeker gets a fixed bottom bar (Jobs,
Courses, Matches, Profile) loaded as a chunk, whose room (--tabbar) is made
before the first paint by a head script so the footer does not jump; the
apply bar and consent banner sit above it. /profile ends 697,966 B
(headroom 2,034). Frontend only: no migration, no API or contract change.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/adr/IISM-ADR-Register.xlsx
+++ b/docs/adr/IISM-ADR-Register.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 75 of 89 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-089.</t>
+          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 76 of 90 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-090.</t>
         </is>
       </c>
     </row>
@@ -225,7 +225,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit b83d88e by scripts/build_adr_register.py.</t>
+          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit 395d925 by scripts/build_adr_register.py.</t>
         </is>
       </c>
     </row>
@@ -261,7 +261,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">75</t>
+          <t xml:space="preserve">76</t>
         </is>
       </c>
     </row>
@@ -6831,8 +6831,80 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-090</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A Job Seeker's Pages Are One Tap Away, the Bottom Bar Is a Chunk Whose Room Is Made Before It Arrives, and the Header Says Where You Are</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">October 2026</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">81</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Active – extends earlier ADR</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Built</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- The page you are on is marked. currentHref (lib/nav.ts, pure) picks the longest link that is the path or a parent of it: /employer/acme/jobs/x/applications is the vacancies page's and /employer/acme/team is the team's, never both. The desktop and mobile nav links are aria-current="page" and drawn filled, so it is not told by colour alone. A link to a place in a page (/#how-it-works) can never be current,…</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted (October 2026). Sprint 81 (Epic B19, BL-19.13). Extends ADR-065 (a page must not jump while it loads), ADR-086 and ADR-087 (tokens, the header graph and the first-load budget) and ADR-089 (the surfaces and the barrel). Frontend only: no migration, no API or contract change (54 operations).</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-065, ADR-086, ADR-087, ADR-089</t>
+        </is>
+      </c>
+      <c r="L91" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M91" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N91" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR header and sprint record in CLAUDE.md / projectContextForMe.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N90"/>
+  <autoFilter ref="A1:N91"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
@@ -7830,8 +7902,30 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint 81</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-090</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A Job Seeker's Pages Are One Tap Away, the Bottom Bar Is a Chunk Whose Room Is Made Before It Arrives, and the Header Says Where You Are</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D34"/>
+  <autoFilter ref="A1:D35"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Sprint 89: back office and static pages on the shared look (BL-19.19, BL-19.20)
ADR-098. Web only; no migration, no API or contract change, no new icon or string.

- cards/grievance-look: one table for a complaint's state, read by the
  operator's queue and the sender's own list
- Overview figures are MetricTiles; verification kind, overdue stages,
  report chips, verified badge and decisions carry a shape
- AudiencePage icons prop; marks on 404, placeholder and legal pages
- Grievance radio rows and legal account link at 44 px
- error.tsx deliberately has no icon (every route's first load)

/admin 697,221 B first load; /profile unchanged at 699,013 (987 B headroom).
1,178 web tests; nothing ran in Playwright (no Chromium).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/adr/IISM-ADR-Register.xlsx
+++ b/docs/adr/IISM-ADR-Register.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 83 of 97 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-097.</t>
+          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 84 of 98 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-098.</t>
         </is>
       </c>
     </row>
@@ -225,7 +225,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit 8b83944 by scripts/build_adr_register.py.</t>
+          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit 4cc0152 by scripts/build_adr_register.py.</t>
         </is>
       </c>
     </row>
@@ -261,7 +261,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">83</t>
+          <t xml:space="preserve">84</t>
         </is>
       </c>
     </row>
@@ -7407,8 +7407,80 @@
         </is>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-098</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Back Office and the Static Pages Say Where Things Stand With a Shape, a Complaint's State Is One Table for Both Its Readers, and the Error Page Has No Picture</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">October 2026</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">89</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F99" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Active – extends earlier ADR</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Built</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- A complaint's state is one table, cards/grievance-look (GRIEVANCE_LOOK: open, acknowledged, resolved, dismissed, each a tone and a shape), read by the operator's queue and by the sender's own list. Before, each had its own tone map and the person's list had no shape at all. - The overview's six figures are MetricTiles (ADR-097), each with a mark and a dash while the number has not arrived, the same shape before…</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted (October 2026). Sprint 89 (Epic B19, BL-19.19 and BL-19.20). Extends ADR-096 and ADR-097 (a state is a word, a shape and a tone, one table per list; a figure has a mark), ADR-083 (the back office's structure and the 44 px floor), ADR-089 (the barrel puts what it names on every route) and ADR-087 (an icon is paid for by every route that loads it). Web only and frontend only: no migration, no API or contract change (54 operations), no new icon, no new message string.</t>
+        </is>
+      </c>
+      <c r="K99" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-083, ADR-087, ADR-089, ADR-096, ADR-097</t>
+        </is>
+      </c>
+      <c r="L99" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M99" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N99" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR header and sprint record in CLAUDE.md / projectContextForMe.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N98"/>
+  <autoFilter ref="A1:N99"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
@@ -8582,8 +8654,30 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint 89</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-098</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Back Office and the Static Pages Say Where Things Stand With a Shape, a Complaint's State Is One Table for Both Its Readers, and the Error Page Has No Picture</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D42"/>
+  <autoFilter ref="A1:D43"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Sprint 90: language and length pass, and the record of Epic B19 (BL-19.25, BL-19.26)
ADR-099. Web only; no migration, no API or contract change, no new icon or string.

- Hindi and Malay checked at 360 px, ordinary size and 200% text, about 90
  page loads across every kind of account: none at ordinary size, ten
  defects at 200%, all fixed (overflow-wrap: anywhere, tab bar, match score
  row, chart labels, applicant chips, profile row buttons, two selects, the
  mobile menu's workspace label)
- src/lib/text-fit.test.ts holds each fix
- build_ui_review.py: nine findings gain a status, stale paragraph rewritten,
  Epic B19 table added; only UI-03 and UI-23 stay open (the owner's)

/profile 699,067 B first load (933 B headroom). 1,187 web tests.
Not run: Playwright, the 52-capture re-run (no Chromium).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/adr/IISM-ADR-Register.xlsx
+++ b/docs/adr/IISM-ADR-Register.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 84 of 98 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-098.</t>
+          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 85 of 99 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-099.</t>
         </is>
       </c>
     </row>
@@ -225,7 +225,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit 4cc0152 by scripts/build_adr_register.py.</t>
+          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit 032a0e6 by scripts/build_adr_register.py.</t>
         </is>
       </c>
     </row>
@@ -261,7 +261,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">84</t>
+          <t xml:space="preserve">85</t>
         </is>
       </c>
     </row>
@@ -7479,8 +7479,80 @@
         </is>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-099</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text That Does Not Fit Is Wrapped or Broken and Never Cut Off, a Page Is Checked at Twice the Size in Every Language, and the Review Says What It Could Not Run</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">October 2026</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">90</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F100" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Active – extends earlier ADR</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Built</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- body { overflow-wrap: anywhere } in globals.css. Not break-word: both break a word that would otherwise overflow, but anywhere also counts the break in the element's minimum width, so a flex item holding "documents/instructions/correspondence" can shrink instead of widening the page. It acts only on a word that would overflow, so ordinary text is unchanged (checked: page heights identical with the rule on and…</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted (October 2026). Sprint 90 (Epic B19, BL-19.25 and BL-19.26). Extends ADR-086 (the type scale: secondary text is 15 px and the floor is 12 px), ADR-077 (accessibility is held by the properties that produce it, and by saying what a test cannot see) and ADR-065 (a page that works at one size is not a page that works). Web only and frontend only: no migration, no API or contract change (54 operations), no new icon, no new message string.</t>
+        </is>
+      </c>
+      <c r="K100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-065, ADR-077, ADR-086</t>
+        </is>
+      </c>
+      <c r="L100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR header and sprint record in CLAUDE.md / projectContextForMe.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N99"/>
+  <autoFilter ref="A1:N100"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
@@ -8676,8 +8748,30 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint 90</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-099</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text That Does Not Fit Is Wrapped or Broken and Never Cut Off, a Page Is Checked at Twice the Size in Every Language, and the Review Says What It Could Not Run</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D43"/>
+  <autoFilter ref="A1:D44"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Sprint 92: the teal theme and two more UX fixes (ADR-101)
Deep teal brand with greys unchanged, success moved to a true green (hue 120),
marigold highlight as decoration-only tokens guarded by a test, assets rendered
from scripts/icons, a public rating needs three, 'Reviewed by our team', the
apply bar's cost line and the filter row's edge fade. Backlog v1.56.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/adr/IISM-ADR-Register.xlsx
+++ b/docs/adr/IISM-ADR-Register.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 86 of 100 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-100.</t>
+          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 87 of 101 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-101.</t>
         </is>
       </c>
     </row>
@@ -225,7 +225,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit bd317c6 by scripts/build_adr_register.py.</t>
+          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit b02587d by scripts/build_adr_register.py.</t>
         </is>
       </c>
     </row>
@@ -261,7 +261,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">86</t>
+          <t xml:space="preserve">87</t>
         </is>
       </c>
     </row>
@@ -7623,8 +7623,80 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-101</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Brand Is Deep Teal, Success Is Moved to a True Green Because Hue Is Measured and Not Guessed, the Highlight Is Decoration Only, and the Public Sees a Score Only From Three Ratings</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">October 2026</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">92</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F102" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Active – extends earlier ADR</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Built</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- Deep teal. Brand ramp #ecf8f8 to #062629, 700 is #0f5c63 (7.7:1 on white, 7.3 on the page, white on it 7.7), dark brand is 400 #35a5ac (6.3:1 on the dark page). The neutral greys are unchanged (the owner kept them), so the address bar's colours, the manifest's background, the offline page and the phone's splash did not move. The mapping of each semantic token to a ramp step is unchanged, which is why every…</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted (October 2026). Sprint 92 (Epic B21, BL-21.2 to BL-21.5; Epic B22, BL-22.4 in part and BL-22.6). Supersedes the part of ADR-086 that fixed brand-700 at the product's old blue (#1f4e79, "the colour the product has always used"); everything else in ADR-086 stands (the look is a token, a ramp step is never a class, text is never translucent). Extends ADR-096 (a state is a word, a shape and a tone). Web and phone, frontend only: no migration, no API or contract change (54 operations), no new icon.</t>
+        </is>
+      </c>
+      <c r="K102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-086, ADR-096</t>
+        </is>
+      </c>
+      <c r="L102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR header and sprint record in CLAUDE.md / projectContextForMe.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N101"/>
+  <autoFilter ref="A1:N102"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
@@ -8864,8 +8936,30 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint 92</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-101</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Brand Is Deep Teal, Success Is Moved to a True Green Because Hue Is Measured and Not Guessed, the Highlight Is Decoration Only, and the Public Sees a Score Only From Three Ratings</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D45"/>
+  <autoFilter ref="A1:D46"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Sprint 92: light by default, and the UX fixes that did not need a colour (ADR-101)
The product is light whatever the device says (the owner's Mac was in dark mode,
so the light page had never been on their screen); dark and 'match the device'
are footer choices, on the web and the phone. A public rating needs three,
verified organisations read 'Reviewed by our team.', the apply bar says what
signing in costs, and the filter row fades at its edge. No palette changed: teal,
aqua and teal-and-marigold were built and looked at and the blue was kept.
Backlog v1.56.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/adr/IISM-ADR-Register.xlsx
+++ b/docs/adr/IISM-ADR-Register.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 86 of 100 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-100.</t>
+          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 87 of 101 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-101.</t>
         </is>
       </c>
     </row>
@@ -225,7 +225,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit bd317c6 by scripts/build_adr_register.py.</t>
+          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit b02587d by scripts/build_adr_register.py.</t>
         </is>
       </c>
     </row>
@@ -261,7 +261,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">86</t>
+          <t xml:space="preserve">87</t>
         </is>
       </c>
     </row>
@@ -7623,8 +7623,80 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-101</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Light Is the Default Because a Dark Computer Hid the Light Page, a Colour Is Judged on the Product Before It Is Chosen, and the Public Sees a Score Only From Three Ratings</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">October 2026</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">92</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F102" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Active</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Built</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- Light is the default, whatever the device says. A visitor who never touches the control gets the light page; dark and "match the device" are choices. lib/theme.ts: a stored value is a choice only if it is dark or system, anything else (or nothing, or storage that throws) is light; choosing light removes the stored value, because light is the absence of one. &lt;html data-theme&gt; is absent for light, dark for dark…</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted (October 2026). Sprint 92 (Epic B21, closed without a palette change; Epic B22, BL-22.4 in part, BL-22.6 and BL-22.10). Supersedes the part of ADR-087 that said the product follows the device's colour scheme until a person chooses; everything else in ADR-087 stands. Web and phone, frontend only: no migration, no API or contract change (54 operations), no new icon. The brand stays blue (#1f4e79, ADR-086).</t>
+        </is>
+      </c>
+      <c r="K102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-086, ADR-087</t>
+        </is>
+      </c>
+      <c r="L102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR header and sprint record in CLAUDE.md / projectContextForMe.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N101"/>
+  <autoFilter ref="A1:N102"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
@@ -8864,8 +8936,30 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint 92</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-101</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Light Is the Default Because a Dark Computer Hid the Light Page, a Colour Is Judged on the Product Before It Is Chosen, and the Public Sees a Score Only From Three Ratings</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D45"/>
+  <autoFilter ref="A1:D46"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Sprint 93: foundations for the training organisation (ADR-102)
ADR-102 designs the dual role (an organisation sells courses, delivers training,
or both; a centre is a child with inherited access and two marks; delivering
another provider's course needs approval). The create-organisation dialog is
fetched on its first click, taking 35,573 B off every route's first load
(/profile 699,148 to 663,575). The operator's verification queue gains search
and a kind filter. Adds the sprint-history spreadsheet. Backlog v1.57.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/adr/IISM-ADR-Register.xlsx
+++ b/docs/adr/IISM-ADR-Register.xlsx
@@ -153,7 +153,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 87 of 101 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-101.</t>
+          <t xml:space="preserve">Yes. It is the live decision record, not a historical artefact. 88 of 102 ADRs are in force or extended by a later one. It is append-only by design: later ADRs refine, extend or supersede earlier ones, and the file is kept up to date through ADR-102.</t>
         </is>
       </c>
     </row>
@@ -225,7 +225,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit b02587d by scripts/build_adr_register.py.</t>
+          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit 25c4637 by scripts/build_adr_register.py.</t>
         </is>
       </c>
     </row>
@@ -261,7 +261,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">87</t>
+          <t xml:space="preserve">88</t>
         </is>
       </c>
     </row>
@@ -7695,8 +7695,80 @@
         </is>
       </c>
     </row>
+    <row r="103">
+      <c r="A103" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-102</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A Training Organisation Sells Courses, Delivers Training, or Both; a Centre Is a Child of the Organisation That Delivers; Delivery of Somebody Else's Course Needs Their Approval</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">October 2026</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">93</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F103" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Active – extends earlier ADR</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Built</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- One organisation, two capabilities. The public word is training organisation; it is stored as tenant_type = "course_provider" (unchanged: a rename strands listings, bulk-upload files and the released phone contract). It has up to two capabilities, stored as two booleans on the tenant, not as two types: publishes_courses ("course provider": publishes courses and receives course-level interest; default true,…</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted as a design (October 2026), to be built in Sprints 94 to 101. Written in Sprint 93 (Epic B18, BL-18.1; Epic B20 is built on it). Extends ADR-026 (a course provider publishes through its own writer), ADR-038 (one identity, many roles: never fork an account), ADR-039 (authorization asks for a permission), ADR-042 (operator authority is outside the tenant model), ADR-068 (a fact about a course that changes is derived) and ADR-069 (every writer of "published" has the one guard). Supersedes nothing. Nothing in this ADR is implemented yet, and Sprint 93 changes no behaviour of it: the sprint makes the room (first-load budget) and the operator's queue search that Sprints 94 to 101 need.</t>
+        </is>
+      </c>
+      <c r="K103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-026, ADR-038, ADR-039, ADR-042, ADR-068, ADR-069</t>
+        </is>
+      </c>
+      <c r="L103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N103" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR header and sprint record in CLAUDE.md / projectContextForMe.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N102"/>
+  <autoFilter ref="A1:N103"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
@@ -8958,8 +9030,30 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sprint 93</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADR-102</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A Training Organisation Sells Courses, Delivers Training, or Both; a Centre Is a Child of the Organisation That Delivers; Delivery of Somebody Else's Course Needs Their Approval</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D46"/>
+  <autoFilter ref="A1:D47"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Sprint 94: capabilities, registration, profile and a public page for the training organisation (ADR-102)
An organisation sells courses, delivers training, or both (two flags on one
organisation, migration 0058, one capability_for function replacing the
organisation-type comparison in require()). Asked for at every way of creating
one and changed by its owner with the server's refusals. A public page
/providers/[slug] shows what it does, its own claims, sectors derived from its
courses and its published courses. Bulk upload notes qualification-like vacancy
titles once per file. Backlog v1.58.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/adr/IISM-ADR-Register.xlsx
+++ b/docs/adr/IISM-ADR-Register.xlsx
@@ -225,7 +225,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit 25c4637 by scripts/build_adr_register.py.</t>
+          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit d5a832d by scripts/build_adr_register.py.</t>
         </is>
       </c>
     </row>
@@ -7713,12 +7713,12 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">93</t>
+          <t xml:space="preserve">94</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0058</t>
         </is>
       </c>
       <c r="F103" s="3" t="inlineStr">
@@ -7743,7 +7743,7 @@
       </c>
       <c r="J103" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted as a design (October 2026), to be built in Sprints 94 to 101. Written in Sprint 93 (Epic B18, BL-18.1; Epic B20 is built on it). Extends ADR-026 (a course provider publishes through its own writer), ADR-038 (one identity, many roles: never fork an account), ADR-039 (authorization asks for a permission), ADR-042 (operator authority is outside the tenant model), ADR-068 (a fact about a course that changes is derived) and ADR-069 (every writer of "published" has the one guard). Supersedes nothing. Nothing in this ADR is implemented yet, and Sprint 93 changes no behaviour of it: the sprint makes the room (first-load budget) and the operator's queue search that Sprints 94 to 101 need.</t>
+          <t xml:space="preserve">Accepted (October 2026); the capabilities, registration, profile and public page are built in Sprint 94 (migration 0058), the rest in Sprints 95 to 101. Written in Sprint 93 (Epic B18, BL-18.1; Epic B20 is built on it). Extends ADR-026 (a course provider publishes through its own writer), ADR-038 (one identity, many roles: never fork an account), ADR-039 (authorization asks for a permission), ADR-042 (operator authority is outside the tenant model), ADR-068 (a fact about a course that changes is derived) and ADR-069 (every writer of "published" has the one guard). Supersedes nothing. Sprint 93 changed no behaviour of it: the sprint made the room (first-load budget) and the operator's queue search that Sprints 94 to 101 need.</t>
         </is>
       </c>
       <c r="K103" s="2" t="inlineStr">
@@ -9033,7 +9033,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint 93</t>
+          <t xml:space="preserve">Sprint 94</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -9048,7 +9048,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0058</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sprint 95: centres, called out by the organisation (ADR-102 in part, migration 0059)
An organisation that delivers training lists its centres: a child tenant
(parent_id RESTRICT, training_centre) with a name, address and resolved place,
added singly or from a checked CSV, edited, closed and reopened. Access is
inherited through one function (centre_for); a centre is never a workspace or
membership. The operator checks a centre's address in the verification queue
(its own mark, removed when a checked address changes; the organisation is
told). Stopping delivery is refused while a centre is open, with a lock against
the race. The public provider page lists open centres; deletion removes
centres first and the previews name them.

2,195 backend / 1,324 web / 816 mobile tests; 45 mutation checks.
Nothing ran in Playwright (no Chromium).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/adr/IISM-ADR-Register.xlsx
+++ b/docs/adr/IISM-ADR-Register.xlsx
@@ -225,7 +225,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit d5a832d by scripts/build_adr_register.py.</t>
+          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit 16f7484 by scripts/build_adr_register.py.</t>
         </is>
       </c>
     </row>
@@ -7743,7 +7743,7 @@
       </c>
       <c r="J103" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted (October 2026); the capabilities, registration, profile and public page are built in Sprint 94 (migration 0058), the rest in Sprints 95 to 101. Written in Sprint 93 (Epic B18, BL-18.1; Epic B20 is built on it). Extends ADR-026 (a course provider publishes through its own writer), ADR-038 (one identity, many roles: never fork an account), ADR-039 (authorization asks for a permission), ADR-042 (operator authority is outside the tenant model), ADR-068 (a fact about a course that changes is derived) and ADR-069 (every writer of "published" has the one guard). Supersedes nothing. Sprint 93 changed no behaviour of it: the sprint made the room (first-load budget) and the operator's queue search that Sprints 94 to 101 need.</t>
+          <t xml:space="preserve">Accepted (October 2026); the capabilities, registration, profile and public page are built in Sprint 94 (migration 0058), centres in Sprint 95 (migration 0059), the rest in Sprints 96 to 101. Written in Sprint 93 (Epic B18, BL-18.1; Epic B20 is built on it). Extends ADR-026 (a course provider publishes through its own writer), ADR-038 (one identity, many roles: never fork an account), ADR-039 (authorization asks for a permission), ADR-042 (operator authority is outside the tenant model), ADR-068 (a fact about a course that changes is derived) and ADR-069 (every writer of "published" has the one guard). Supersedes nothing. Sprint 93 changed no behaviour of it: the sprint made the room (first-load budget) and the operator's queue search that Sprints 94 to 101 need.</t>
         </is>
       </c>
       <c r="K103" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sprint 96: centre staff and the fourth kind (ADR-102 in part, migration 0060)
The person who runs a training centre is a manager: a membership on the centre's
own row, asked in by the organisation's owners and admins through the existing
invitation flow (a mail naming the centre and the organisation). Only the
organisation decides who runs a centre; the cap of ten managers is counted under
the ownership lock on the centre's row (race test). A manager reaches their
centre and nothing of the organisation: no ORG_READ, and a route sweep as a
manager holds it. A manager's erasure leaves the centre alone. The header,
switcher, welcome card and invitation page handle the fourth kind with no layout
change; /employer/[org] loads a third workspace chunk only for a centre.

2,223 backend / 1,352 web / 816 mobile tests; 34 mutation checks.
Nothing ran in Playwright (no Chromium).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/adr/IISM-ADR-Register.xlsx
+++ b/docs/adr/IISM-ADR-Register.xlsx
@@ -225,7 +225,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit 16f7484 by scripts/build_adr_register.py.</t>
+          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit d94145e by scripts/build_adr_register.py.</t>
         </is>
       </c>
     </row>
@@ -7743,7 +7743,7 @@
       </c>
       <c r="J103" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted (October 2026); the capabilities, registration, profile and public page are built in Sprint 94 (migration 0058), centres in Sprint 95 (migration 0059), the rest in Sprints 96 to 101. Written in Sprint 93 (Epic B18, BL-18.1; Epic B20 is built on it). Extends ADR-026 (a course provider publishes through its own writer), ADR-038 (one identity, many roles: never fork an account), ADR-039 (authorization asks for a permission), ADR-042 (operator authority is outside the tenant model), ADR-068 (a fact about a course that changes is derived) and ADR-069 (every writer of "published" has the one guard). Supersedes nothing. Sprint 93 changed no behaviour of it: the sprint made the room (first-load budget) and the operator's queue search that Sprints 94 to 101 need.</t>
+          <t xml:space="preserve">Accepted (October 2026); the capabilities, registration, profile and public page are built in Sprint 94 (migration 0058), centres in Sprint 95 (migration 0059), centre staff in Sprint 96 (migration 0060), the rest in Sprints 97 to 101. Written in Sprint 93 (Epic B18, BL-18.1; Epic B20 is built on it). Extends ADR-026 (a course provider publishes through its own writer), ADR-038 (one identity, many roles: never fork an account), ADR-039 (authorization asks for a permission), ADR-042 (operator authority is outside the tenant model), ADR-068 (a fact about a course that changes is derived) and ADR-069 (every writer of "published" has the one guard). Supersedes nothing. Sprint 93 changed no behaviour of it: the sprint made the room (first-load budget) and the operator's queue search that Sprints 94 to 101 need.</t>
         </is>
       </c>
       <c r="K103" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sprint 98: batches and the batch card (ADR-103, BL-18.5)
A delivering organisation plans, publishes, changes and cancels a batch of a course
it owns or is authorised to deliver. Phase is derived; authorisation is asked at
creation and publication under a share lock revoke also takes; revoking cancels
batches not yet started and tells learners; centres and courses cannot go from
under a live batch. Built on ADR-103's recommendations (owner's three decisions
unanswered). Also: schema-name clash guard, grid-cols-1 fix for 200% Hindi.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/adr/IISM-ADR-Register.xlsx
+++ b/docs/adr/IISM-ADR-Register.xlsx
@@ -225,7 +225,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit 09d3f43 by scripts/build_adr_register.py.</t>
+          <t xml:space="preserve">From docs/adr/architecture-decisions.md at commit 8b89bb5 by scripts/build_adr_register.py.</t>
         </is>
       </c>
     </row>
@@ -7780,12 +7780,12 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">October 2026</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">97</t>
+          <t xml:space="preserve">98</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -7815,7 +7815,7 @@
       </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed (October 2026), written in Sprint 97 (Epic B18, BL-18.5; Epic B20 is built on it). The delivery authorisations it depends on are built (ADR-102, migration 0061); the batch itself is Sprint 98. Three decisions are the owner's and are written here as recommendations, marked below; nothing in Sprint 98 is built on them until the owner confirms or changes them. Extends ADR-102 (centres, authorisations), ADR-068 (a fact about a course that changes is derived), ADR-071 (a join table, never a foreign key into a module that may not be imported), ADR-082 (require_not_paused guards every writer of contact) and ADR-025/047 (the enrolment metric).</t>
+          <t xml:space="preserve">Proposed (October 2026; the batch itself built in Sprint 98, see the end), written in Sprint 97 (Epic B18, BL-18.5; Epic B20 is built on it). The delivery authorisations it depends on are built (ADR-102, migration 0061); the batch itself is Sprint 98. Three decisions are the owner's and are written here as recommendations, marked below; nothing in Sprint 98 is built on them until the owner confirms or changes them. Extends ADR-102 (centres, authorisations), ADR-068 (a fact about a course that changes is derived), ADR-071 (a join table, never a foreign key into a module that may not be imported), ADR-082 (require_not_paused guards every writer of contact) and ADR-025/047 (the enrolment metric).</t>
         </is>
       </c>
       <c r="K104" s="2" t="inlineStr">
@@ -9127,7 +9127,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint 97</t>
+          <t xml:space="preserve">Sprint 98</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">

</xml_diff>